<commit_message>
Match 2026 plan workbook to requested table
</commit_message>
<xml_diff>
--- a/templates/計画_2026年.xlsx
+++ b/templates/計画_2026年.xlsx
@@ -46,8 +46,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -415,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N50"/>
+  <dimension ref="A1:N46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -526,43 +527,43 @@
           <t>阿波尾鶏</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="1" t="n">
         <v>54600</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C5" s="1" t="n">
         <v>52000</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" s="1" t="n">
         <v>57200</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E5" s="1" t="n">
         <v>54600</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F5" s="1" t="n">
         <v>54600</v>
       </c>
-      <c r="G5" t="n">
+      <c r="G5" s="1" t="n">
         <v>57200</v>
       </c>
-      <c r="H5" t="n">
+      <c r="H5" s="1" t="n">
         <v>54600</v>
       </c>
-      <c r="I5" t="n">
+      <c r="I5" s="1" t="n">
         <v>62000</v>
       </c>
-      <c r="J5" t="n">
+      <c r="J5" s="1" t="n">
         <v>62000</v>
       </c>
-      <c r="K5" t="n">
+      <c r="K5" s="1" t="n">
         <v>71300</v>
       </c>
-      <c r="L5" t="n">
+      <c r="L5" s="1" t="n">
         <v>65100</v>
       </c>
-      <c r="M5" t="n">
+      <c r="M5" s="1" t="n">
         <v>79000</v>
       </c>
-      <c r="N5" t="n">
+      <c r="N5" s="1" t="n">
         <v>724200</v>
       </c>
     </row>
@@ -572,31 +573,35 @@
           <t>赤どり</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" s="1" t="n">
         <v>84000</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C6" s="1" t="n">
         <v>80000</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D6" s="1" t="n">
         <v>88000</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E6" s="1" t="n">
         <v>84000</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F6" s="1" t="n">
         <v>84000</v>
       </c>
-      <c r="G6" t="n">
+      <c r="G6" s="1" t="n">
         <v>88000</v>
       </c>
-      <c r="H6" t="n">
+      <c r="H6" s="1" t="n">
         <v>84000</v>
       </c>
-      <c r="I6" t="n">
+      <c r="I6" s="1" t="n">
         <v>80000</v>
       </c>
-      <c r="N6" t="n">
+      <c r="J6" s="1" t="n"/>
+      <c r="K6" s="1" t="n"/>
+      <c r="L6" s="1" t="n"/>
+      <c r="M6" s="1" t="n"/>
+      <c r="N6" s="1" t="n">
         <v>672000</v>
       </c>
     </row>
@@ -606,43 +611,43 @@
           <t>地養鳥</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B7" s="1" t="n">
         <v>336000</v>
       </c>
-      <c r="C7" t="n">
+      <c r="C7" s="1" t="n">
         <v>320000</v>
       </c>
-      <c r="D7" t="n">
+      <c r="D7" s="1" t="n">
         <v>352000</v>
       </c>
-      <c r="E7" t="n">
+      <c r="E7" s="1" t="n">
         <v>336000</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F7" s="1" t="n">
         <v>336000</v>
       </c>
-      <c r="G7" t="n">
+      <c r="G7" s="1" t="n">
         <v>352000</v>
       </c>
-      <c r="H7" t="n">
+      <c r="H7" s="1" t="n">
         <v>336000</v>
       </c>
-      <c r="I7" t="n">
+      <c r="I7" s="1" t="n">
         <v>320000</v>
       </c>
-      <c r="J7" t="n">
+      <c r="J7" s="1" t="n">
         <v>320000</v>
       </c>
-      <c r="K7" t="n">
+      <c r="K7" s="1" t="n">
         <v>368000</v>
       </c>
-      <c r="L7" t="n">
+      <c r="L7" s="1" t="n">
         <v>336000</v>
       </c>
-      <c r="M7" t="n">
+      <c r="M7" s="1" t="n">
         <v>400000</v>
       </c>
-      <c r="N7" t="n">
+      <c r="N7" s="1" t="n">
         <v>4112000</v>
       </c>
     </row>
@@ -652,43 +657,43 @@
           <t>ブロイラー</t>
         </is>
       </c>
-      <c r="B8" t="n">
+      <c r="B8" s="1" t="n">
         <v>250900</v>
       </c>
-      <c r="C8" t="n">
+      <c r="C8" s="1" t="n">
         <v>218000</v>
       </c>
-      <c r="D8" t="n">
+      <c r="D8" s="1" t="n">
         <v>243800</v>
       </c>
-      <c r="E8" t="n">
+      <c r="E8" s="1" t="n">
         <v>263400</v>
       </c>
-      <c r="F8" t="n">
+      <c r="F8" s="1" t="n">
         <v>231900</v>
       </c>
-      <c r="G8" t="n">
+      <c r="G8" s="1" t="n">
         <v>210800</v>
       </c>
-      <c r="H8" t="n">
+      <c r="H8" s="1" t="n">
         <v>233400</v>
       </c>
-      <c r="I8" t="n">
+      <c r="I8" s="1" t="n">
         <v>197500</v>
       </c>
-      <c r="J8" t="n">
+      <c r="J8" s="1" t="n">
         <v>279500</v>
       </c>
-      <c r="K8" t="n">
+      <c r="K8" s="1" t="n">
         <v>317200</v>
       </c>
-      <c r="L8" t="n">
+      <c r="L8" s="1" t="n">
         <v>324400</v>
       </c>
-      <c r="M8" t="n">
+      <c r="M8" s="1" t="n">
         <v>342500</v>
       </c>
-      <c r="N8" t="n">
+      <c r="N8" s="1" t="n">
         <v>3113300</v>
       </c>
     </row>
@@ -698,43 +703,43 @@
           <t>ブロイラー（外部）</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="B9" s="1" t="n">
         <v>62000</v>
       </c>
-      <c r="C9" t="n">
+      <c r="C9" s="1" t="n">
         <v>60000</v>
       </c>
-      <c r="D9" t="n">
+      <c r="D9" s="1" t="n">
         <v>62000</v>
       </c>
-      <c r="E9" t="n">
+      <c r="E9" s="1" t="n">
         <v>60000</v>
       </c>
-      <c r="F9" t="n">
+      <c r="F9" s="1" t="n">
         <v>60000</v>
       </c>
-      <c r="G9" t="n">
+      <c r="G9" s="1" t="n">
         <v>62000</v>
       </c>
-      <c r="H9" t="n">
+      <c r="H9" s="1" t="n">
         <v>58500</v>
       </c>
-      <c r="I9" t="n">
+      <c r="I9" s="1" t="n">
         <v>60500</v>
       </c>
-      <c r="J9" t="n">
+      <c r="J9" s="1" t="n">
         <v>58500</v>
       </c>
-      <c r="K9" t="n">
+      <c r="K9" s="1" t="n">
         <v>60000</v>
       </c>
-      <c r="L9" t="n">
+      <c r="L9" s="1" t="n">
         <v>62000</v>
       </c>
-      <c r="M9" t="n">
+      <c r="M9" s="1" t="n">
         <v>64000</v>
       </c>
-      <c r="N9" t="n">
+      <c r="N9" s="1" t="n">
         <v>729500</v>
       </c>
     </row>
@@ -744,43 +749,43 @@
           <t>合計</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="B10" s="1" t="n">
         <v>787500</v>
       </c>
-      <c r="C10" t="n">
+      <c r="C10" s="1" t="n">
         <v>730000</v>
       </c>
-      <c r="D10" t="n">
+      <c r="D10" s="1" t="n">
         <v>803000</v>
       </c>
-      <c r="E10" t="n">
+      <c r="E10" s="1" t="n">
         <v>798000</v>
       </c>
-      <c r="F10" t="n">
+      <c r="F10" s="1" t="n">
         <v>766500</v>
       </c>
-      <c r="G10" t="n">
+      <c r="G10" s="1" t="n">
         <v>770000</v>
       </c>
-      <c r="H10" t="n">
+      <c r="H10" s="1" t="n">
         <v>766500</v>
       </c>
-      <c r="I10" t="n">
+      <c r="I10" s="1" t="n">
         <v>720000</v>
       </c>
-      <c r="J10" t="n">
+      <c r="J10" s="1" t="n">
         <v>720000</v>
       </c>
-      <c r="K10" t="n">
+      <c r="K10" s="1" t="n">
         <v>816500</v>
       </c>
-      <c r="L10" t="n">
+      <c r="L10" s="1" t="n">
         <v>787500</v>
       </c>
-      <c r="M10" t="n">
+      <c r="M10" s="1" t="n">
         <v>885500</v>
       </c>
-      <c r="N10" t="n">
+      <c r="N10" s="1" t="n">
         <v>9351000</v>
       </c>
     </row>
@@ -869,43 +874,43 @@
           <t>阿波尾鶏</t>
         </is>
       </c>
-      <c r="B14" t="n">
+      <c r="B14" s="1" t="n">
         <v>53508</v>
       </c>
-      <c r="C14" t="n">
+      <c r="C14" s="1" t="n">
         <v>50960</v>
       </c>
-      <c r="D14" t="n">
+      <c r="D14" s="1" t="n">
         <v>56056</v>
       </c>
-      <c r="E14" t="n">
+      <c r="E14" s="1" t="n">
         <v>53508</v>
       </c>
-      <c r="F14" t="n">
+      <c r="F14" s="1" t="n">
         <v>53508</v>
       </c>
-      <c r="G14" t="n">
+      <c r="G14" s="1" t="n">
         <v>56056</v>
       </c>
-      <c r="H14" t="n">
+      <c r="H14" s="1" t="n">
         <v>53508</v>
       </c>
-      <c r="I14" t="n">
+      <c r="I14" s="1" t="n">
         <v>60760</v>
       </c>
-      <c r="J14" t="n">
+      <c r="J14" s="1" t="n">
         <v>60760</v>
       </c>
-      <c r="K14" t="n">
+      <c r="K14" s="1" t="n">
         <v>69874</v>
       </c>
-      <c r="L14" t="n">
+      <c r="L14" s="1" t="n">
         <v>63798</v>
       </c>
-      <c r="M14" t="n">
+      <c r="M14" s="1" t="n">
         <v>77420</v>
       </c>
-      <c r="N14" t="n">
+      <c r="N14" s="1" t="n">
         <v>709716</v>
       </c>
     </row>
@@ -915,31 +920,35 @@
           <t>赤どり</t>
         </is>
       </c>
-      <c r="B15" t="n">
+      <c r="B15" s="1" t="n">
         <v>81480</v>
       </c>
-      <c r="C15" t="n">
+      <c r="C15" s="1" t="n">
         <v>77600</v>
       </c>
-      <c r="D15" t="n">
+      <c r="D15" s="1" t="n">
         <v>85360</v>
       </c>
-      <c r="E15" t="n">
+      <c r="E15" s="1" t="n">
         <v>81480</v>
       </c>
-      <c r="F15" t="n">
+      <c r="F15" s="1" t="n">
         <v>81480</v>
       </c>
-      <c r="G15" t="n">
+      <c r="G15" s="1" t="n">
         <v>85360</v>
       </c>
-      <c r="H15" t="n">
+      <c r="H15" s="1" t="n">
         <v>81480</v>
       </c>
-      <c r="I15" t="n">
+      <c r="I15" s="1" t="n">
         <v>77600</v>
       </c>
-      <c r="N15" t="n">
+      <c r="J15" s="1" t="n"/>
+      <c r="K15" s="1" t="n"/>
+      <c r="L15" s="1" t="n"/>
+      <c r="M15" s="1" t="n"/>
+      <c r="N15" s="1" t="n">
         <v>651840</v>
       </c>
     </row>
@@ -949,43 +958,43 @@
           <t>地養鳥</t>
         </is>
       </c>
-      <c r="B16" t="n">
+      <c r="B16" s="1" t="n">
         <v>329280</v>
       </c>
-      <c r="C16" t="n">
+      <c r="C16" s="1" t="n">
         <v>313600</v>
       </c>
-      <c r="D16" t="n">
+      <c r="D16" s="1" t="n">
         <v>344960</v>
       </c>
-      <c r="E16" t="n">
+      <c r="E16" s="1" t="n">
         <v>329280</v>
       </c>
-      <c r="F16" t="n">
+      <c r="F16" s="1" t="n">
         <v>329280</v>
       </c>
-      <c r="G16" t="n">
+      <c r="G16" s="1" t="n">
         <v>344960</v>
       </c>
-      <c r="H16" t="n">
+      <c r="H16" s="1" t="n">
         <v>329280</v>
       </c>
-      <c r="I16" t="n">
+      <c r="I16" s="1" t="n">
         <v>313600</v>
       </c>
-      <c r="J16" t="n">
+      <c r="J16" s="1" t="n">
         <v>313600</v>
       </c>
-      <c r="K16" t="n">
+      <c r="K16" s="1" t="n">
         <v>360640</v>
       </c>
-      <c r="L16" t="n">
+      <c r="L16" s="1" t="n">
         <v>329280</v>
       </c>
-      <c r="M16" t="n">
+      <c r="M16" s="1" t="n">
         <v>392000</v>
       </c>
-      <c r="N16" t="n">
+      <c r="N16" s="1" t="n">
         <v>4029760</v>
       </c>
     </row>
@@ -995,43 +1004,43 @@
           <t>ブロイラー</t>
         </is>
       </c>
-      <c r="B17" t="n">
+      <c r="B17" s="1" t="n">
         <v>245882</v>
       </c>
-      <c r="C17" t="n">
+      <c r="C17" s="1" t="n">
         <v>213640</v>
       </c>
-      <c r="D17" t="n">
+      <c r="D17" s="1" t="n">
         <v>238924</v>
       </c>
-      <c r="E17" t="n">
+      <c r="E17" s="1" t="n">
         <v>258132</v>
       </c>
-      <c r="F17" t="n">
+      <c r="F17" s="1" t="n">
         <v>227262</v>
       </c>
-      <c r="G17" t="n">
+      <c r="G17" s="1" t="n">
         <v>206584</v>
       </c>
-      <c r="H17" t="n">
+      <c r="H17" s="1" t="n">
         <v>228732</v>
       </c>
-      <c r="I17" t="n">
+      <c r="I17" s="1" t="n">
         <v>193550</v>
       </c>
-      <c r="J17" t="n">
+      <c r="J17" s="1" t="n">
         <v>273910</v>
       </c>
-      <c r="K17" t="n">
+      <c r="K17" s="1" t="n">
         <v>310856</v>
       </c>
-      <c r="L17" t="n">
+      <c r="L17" s="1" t="n">
         <v>317912</v>
       </c>
-      <c r="M17" t="n">
+      <c r="M17" s="1" t="n">
         <v>335650</v>
       </c>
-      <c r="N17" t="n">
+      <c r="N17" s="1" t="n">
         <v>3051034</v>
       </c>
     </row>
@@ -1041,43 +1050,43 @@
           <t>ブロイラー（外部）</t>
         </is>
       </c>
-      <c r="B18" t="n">
+      <c r="B18" s="1" t="n">
         <v>60760</v>
       </c>
-      <c r="C18" t="n">
+      <c r="C18" s="1" t="n">
         <v>58800</v>
       </c>
-      <c r="D18" t="n">
+      <c r="D18" s="1" t="n">
         <v>60760</v>
       </c>
-      <c r="E18" t="n">
+      <c r="E18" s="1" t="n">
         <v>58800</v>
       </c>
-      <c r="F18" t="n">
+      <c r="F18" s="1" t="n">
         <v>58800</v>
       </c>
-      <c r="G18" t="n">
+      <c r="G18" s="1" t="n">
         <v>60760</v>
       </c>
-      <c r="H18" t="n">
+      <c r="H18" s="1" t="n">
         <v>57330</v>
       </c>
-      <c r="I18" t="n">
+      <c r="I18" s="1" t="n">
         <v>59290</v>
       </c>
-      <c r="J18" t="n">
+      <c r="J18" s="1" t="n">
         <v>57330</v>
       </c>
-      <c r="K18" t="n">
+      <c r="K18" s="1" t="n">
         <v>58800</v>
       </c>
-      <c r="L18" t="n">
+      <c r="L18" s="1" t="n">
         <v>60760</v>
       </c>
-      <c r="M18" t="n">
+      <c r="M18" s="1" t="n">
         <v>62720</v>
       </c>
-      <c r="N18" t="n">
+      <c r="N18" s="1" t="n">
         <v>714910</v>
       </c>
     </row>
@@ -1087,43 +1096,43 @@
           <t>合計</t>
         </is>
       </c>
-      <c r="B19" t="n">
+      <c r="B19" s="1" t="n">
         <v>770910</v>
       </c>
-      <c r="C19" t="n">
+      <c r="C19" s="1" t="n">
         <v>714600</v>
       </c>
-      <c r="D19" t="n">
+      <c r="D19" s="1" t="n">
         <v>786060</v>
       </c>
-      <c r="E19" t="n">
+      <c r="E19" s="1" t="n">
         <v>781200</v>
       </c>
-      <c r="F19" t="n">
+      <c r="F19" s="1" t="n">
         <v>750330</v>
       </c>
-      <c r="G19" t="n">
+      <c r="G19" s="1" t="n">
         <v>753720</v>
       </c>
-      <c r="H19" t="n">
+      <c r="H19" s="1" t="n">
         <v>750330</v>
       </c>
-      <c r="I19" t="n">
+      <c r="I19" s="1" t="n">
         <v>704800</v>
       </c>
-      <c r="J19" t="n">
+      <c r="J19" s="1" t="n">
         <v>705600</v>
       </c>
-      <c r="K19" t="n">
+      <c r="K19" s="1" t="n">
         <v>800170</v>
       </c>
-      <c r="L19" t="n">
+      <c r="L19" s="1" t="n">
         <v>771750</v>
       </c>
-      <c r="M19" t="n">
+      <c r="M19" s="1" t="n">
         <v>867790</v>
       </c>
-      <c r="N19" t="n">
+      <c r="N19" s="1" t="n">
         <v>9157260</v>
       </c>
     </row>
@@ -1212,43 +1221,43 @@
           <t>阿波尾鶏</t>
         </is>
       </c>
-      <c r="B23" t="n">
+      <c r="B23" s="1" t="n">
         <v>187278</v>
       </c>
-      <c r="C23" t="n">
+      <c r="C23" s="1" t="n">
         <v>178360</v>
       </c>
-      <c r="D23" t="n">
+      <c r="D23" s="1" t="n">
         <v>196196</v>
       </c>
-      <c r="E23" t="n">
+      <c r="E23" s="1" t="n">
         <v>187278</v>
       </c>
-      <c r="F23" t="n">
+      <c r="F23" s="1" t="n">
         <v>187278</v>
       </c>
-      <c r="G23" t="n">
+      <c r="G23" s="1" t="n">
         <v>196196</v>
       </c>
-      <c r="H23" t="n">
+      <c r="H23" s="1" t="n">
         <v>181927</v>
       </c>
-      <c r="I23" t="n">
+      <c r="I23" s="1" t="n">
         <v>206584</v>
       </c>
-      <c r="J23" t="n">
+      <c r="J23" s="1" t="n">
         <v>212660</v>
       </c>
-      <c r="K23" t="n">
+      <c r="K23" s="1" t="n">
         <v>244559</v>
       </c>
-      <c r="L23" t="n">
+      <c r="L23" s="1" t="n">
         <v>223293</v>
       </c>
-      <c r="M23" t="n">
+      <c r="M23" s="1" t="n">
         <v>270970</v>
       </c>
-      <c r="N23" t="n">
+      <c r="N23" s="1" t="n">
         <v>2472579</v>
       </c>
     </row>
@@ -1258,31 +1267,35 @@
           <t>赤どり</t>
         </is>
       </c>
-      <c r="B24" t="n">
+      <c r="B24" s="1" t="n">
         <v>252588</v>
       </c>
-      <c r="C24" t="n">
+      <c r="C24" s="1" t="n">
         <v>240560</v>
       </c>
-      <c r="D24" t="n">
+      <c r="D24" s="1" t="n">
         <v>264616</v>
       </c>
-      <c r="E24" t="n">
+      <c r="E24" s="1" t="n">
         <v>252588</v>
       </c>
-      <c r="F24" t="n">
+      <c r="F24" s="1" t="n">
         <v>252588</v>
       </c>
-      <c r="G24" t="n">
+      <c r="G24" s="1" t="n">
         <v>264616</v>
       </c>
-      <c r="H24" t="n">
+      <c r="H24" s="1" t="n">
         <v>252588</v>
       </c>
-      <c r="I24" t="n">
+      <c r="I24" s="1" t="n">
         <v>240560</v>
       </c>
-      <c r="N24" t="n">
+      <c r="J24" s="1" t="n"/>
+      <c r="K24" s="1" t="n"/>
+      <c r="L24" s="1" t="n"/>
+      <c r="M24" s="1" t="n"/>
+      <c r="N24" s="1" t="n">
         <v>2020704</v>
       </c>
     </row>
@@ -1292,43 +1305,43 @@
           <t>地養鳥</t>
         </is>
       </c>
-      <c r="B25" t="n">
+      <c r="B25" s="1" t="n">
         <v>987840</v>
       </c>
-      <c r="C25" t="n">
+      <c r="C25" s="1" t="n">
         <v>940800</v>
       </c>
-      <c r="D25" t="n">
+      <c r="D25" s="1" t="n">
         <v>1034880</v>
       </c>
-      <c r="E25" t="n">
+      <c r="E25" s="1" t="n">
         <v>987840</v>
       </c>
-      <c r="F25" t="n">
+      <c r="F25" s="1" t="n">
         <v>987840</v>
       </c>
-      <c r="G25" t="n">
+      <c r="G25" s="1" t="n">
         <v>1034880</v>
       </c>
-      <c r="H25" t="n">
+      <c r="H25" s="1" t="n">
         <v>971376</v>
       </c>
-      <c r="I25" t="n">
+      <c r="I25" s="1" t="n">
         <v>925120</v>
       </c>
-      <c r="J25" t="n">
+      <c r="J25" s="1" t="n">
         <v>925120</v>
       </c>
-      <c r="K25" t="n">
+      <c r="K25" s="1" t="n">
         <v>1081920</v>
       </c>
-      <c r="L25" t="n">
+      <c r="L25" s="1" t="n">
         <v>987840</v>
       </c>
-      <c r="M25" t="n">
+      <c r="M25" s="1" t="n">
         <v>1176000</v>
       </c>
-      <c r="N25" t="n">
+      <c r="N25" s="1" t="n">
         <v>12041456</v>
       </c>
     </row>
@@ -1338,43 +1351,43 @@
           <t>ブロイラー</t>
         </is>
       </c>
-      <c r="B26" t="n">
+      <c r="B26" s="1" t="n">
         <v>749940</v>
       </c>
-      <c r="C26" t="n">
+      <c r="C26" s="1" t="n">
         <v>651602</v>
       </c>
-      <c r="D26" t="n">
+      <c r="D26" s="1" t="n">
         <v>728718</v>
       </c>
-      <c r="E26" t="n">
+      <c r="E26" s="1" t="n">
         <v>787303</v>
       </c>
-      <c r="F26" t="n">
+      <c r="F26" s="1" t="n">
         <v>693149</v>
       </c>
-      <c r="G26" t="n">
+      <c r="G26" s="1" t="n">
         <v>630081</v>
       </c>
-      <c r="H26" t="n">
+      <c r="H26" s="1" t="n">
         <v>686196</v>
       </c>
-      <c r="I26" t="n">
+      <c r="I26" s="1" t="n">
         <v>580650</v>
       </c>
-      <c r="J26" t="n">
+      <c r="J26" s="1" t="n">
         <v>821730</v>
       </c>
-      <c r="K26" t="n">
+      <c r="K26" s="1" t="n">
         <v>948111</v>
       </c>
-      <c r="L26" t="n">
+      <c r="L26" s="1" t="n">
         <v>969632</v>
       </c>
-      <c r="M26" t="n">
+      <c r="M26" s="1" t="n">
         <v>1023733</v>
       </c>
-      <c r="N26" t="n">
+      <c r="N26" s="1" t="n">
         <v>9270844</v>
       </c>
     </row>
@@ -1384,43 +1397,43 @@
           <t>ブロイラー（外部）</t>
         </is>
       </c>
-      <c r="B27" t="n">
+      <c r="B27" s="1" t="n">
         <v>185318</v>
       </c>
-      <c r="C27" t="n">
+      <c r="C27" s="1" t="n">
         <v>179340</v>
       </c>
-      <c r="D27" t="n">
+      <c r="D27" s="1" t="n">
         <v>185318</v>
       </c>
-      <c r="E27" t="n">
+      <c r="E27" s="1" t="n">
         <v>179340</v>
       </c>
-      <c r="F27" t="n">
+      <c r="F27" s="1" t="n">
         <v>179340</v>
       </c>
-      <c r="G27" t="n">
+      <c r="G27" s="1" t="n">
         <v>185318</v>
       </c>
-      <c r="H27" t="n">
+      <c r="H27" s="1" t="n">
         <v>171990</v>
       </c>
-      <c r="I27" t="n">
+      <c r="I27" s="1" t="n">
         <v>177870</v>
       </c>
-      <c r="J27" t="n">
+      <c r="J27" s="1" t="n">
         <v>171990</v>
       </c>
-      <c r="K27" t="n">
+      <c r="K27" s="1" t="n">
         <v>179340</v>
       </c>
-      <c r="L27" t="n">
+      <c r="L27" s="1" t="n">
         <v>185318</v>
       </c>
-      <c r="M27" t="n">
+      <c r="M27" s="1" t="n">
         <v>191296</v>
       </c>
-      <c r="N27" t="n">
+      <c r="N27" s="1" t="n">
         <v>2171778</v>
       </c>
     </row>
@@ -1430,43 +1443,43 @@
           <t>合計</t>
         </is>
       </c>
-      <c r="B28" t="n">
+      <c r="B28" s="1" t="n">
         <v>2362964</v>
       </c>
-      <c r="C28" t="n">
+      <c r="C28" s="1" t="n">
         <v>2190662</v>
       </c>
-      <c r="D28" t="n">
+      <c r="D28" s="1" t="n">
         <v>2409728</v>
       </c>
-      <c r="E28" t="n">
+      <c r="E28" s="1" t="n">
         <v>2394349</v>
       </c>
-      <c r="F28" t="n">
+      <c r="F28" s="1" t="n">
         <v>2300195</v>
       </c>
-      <c r="G28" t="n">
+      <c r="G28" s="1" t="n">
         <v>2311091</v>
       </c>
-      <c r="H28" t="n">
+      <c r="H28" s="1" t="n">
         <v>2264077</v>
       </c>
-      <c r="I28" t="n">
+      <c r="I28" s="1" t="n">
         <v>2130784</v>
       </c>
-      <c r="J28" t="n">
+      <c r="J28" s="1" t="n">
         <v>2131500</v>
       </c>
-      <c r="K28" t="n">
+      <c r="K28" s="1" t="n">
         <v>2453930</v>
       </c>
-      <c r="L28" t="n">
+      <c r="L28" s="1" t="n">
         <v>2366083</v>
       </c>
-      <c r="M28" t="n">
+      <c r="M28" s="1" t="n">
         <v>2661999</v>
       </c>
-      <c r="N28" t="n">
+      <c r="N28" s="1" t="n">
         <v>27977361</v>
       </c>
     </row>
@@ -1555,43 +1568,43 @@
           <t>阿波尾鶏</t>
         </is>
       </c>
-      <c r="B32" s="1" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="C32" s="1" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="D32" s="1" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="E32" s="1" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="F32" s="1" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="G32" s="1" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="H32" s="1" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="I32" s="1" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="J32" s="1" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="K32" s="1" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="L32" s="1" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="M32" s="1" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="N32" s="1" t="n">
+      <c r="B32" s="2" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="C32" s="2" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="D32" s="2" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="E32" s="2" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="F32" s="2" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="G32" s="2" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="H32" s="2" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="I32" s="2" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="J32" s="2" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="K32" s="2" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="L32" s="2" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="M32" s="2" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="N32" s="2" t="n">
         <v>0.98</v>
       </c>
     </row>
@@ -1601,43 +1614,43 @@
           <t>赤どり</t>
         </is>
       </c>
-      <c r="B33" s="1" t="n">
+      <c r="B33" s="2" t="n">
         <v>0.97</v>
       </c>
-      <c r="C33" s="1" t="n">
+      <c r="C33" s="2" t="n">
         <v>0.97</v>
       </c>
-      <c r="D33" s="1" t="n">
+      <c r="D33" s="2" t="n">
         <v>0.97</v>
       </c>
-      <c r="E33" s="1" t="n">
+      <c r="E33" s="2" t="n">
         <v>0.97</v>
       </c>
-      <c r="F33" s="1" t="n">
+      <c r="F33" s="2" t="n">
         <v>0.97</v>
       </c>
-      <c r="G33" s="1" t="n">
+      <c r="G33" s="2" t="n">
         <v>0.97</v>
       </c>
-      <c r="H33" s="1" t="n">
+      <c r="H33" s="2" t="n">
         <v>0.97</v>
       </c>
-      <c r="I33" s="1" t="n">
+      <c r="I33" s="2" t="n">
         <v>0.97</v>
       </c>
-      <c r="J33" s="1" t="n">
+      <c r="J33" s="2" t="n">
         <v>0.97</v>
       </c>
-      <c r="K33" s="1" t="n">
+      <c r="K33" s="2" t="n">
         <v>0.97</v>
       </c>
-      <c r="L33" s="1" t="n">
+      <c r="L33" s="2" t="n">
         <v>0.97</v>
       </c>
-      <c r="M33" s="1" t="n">
+      <c r="M33" s="2" t="n">
         <v>0.97</v>
       </c>
-      <c r="N33" s="1" t="n">
+      <c r="N33" s="2" t="n">
         <v>0.97</v>
       </c>
     </row>
@@ -1647,43 +1660,43 @@
           <t>地養鳥</t>
         </is>
       </c>
-      <c r="B34" s="1" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="C34" s="1" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="D34" s="1" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="E34" s="1" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="F34" s="1" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="G34" s="1" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="H34" s="1" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="I34" s="1" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="J34" s="1" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="K34" s="1" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="L34" s="1" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="M34" s="1" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="N34" s="1" t="n">
+      <c r="B34" s="2" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="C34" s="2" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="D34" s="2" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="E34" s="2" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="F34" s="2" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="G34" s="2" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="H34" s="2" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="I34" s="2" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="J34" s="2" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="K34" s="2" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="L34" s="2" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="M34" s="2" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="N34" s="2" t="n">
         <v>0.98</v>
       </c>
     </row>
@@ -1693,43 +1706,43 @@
           <t>ブロイラー</t>
         </is>
       </c>
-      <c r="B35" s="1" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="C35" s="1" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="D35" s="1" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="E35" s="1" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="F35" s="1" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="G35" s="1" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="H35" s="1" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="I35" s="1" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="J35" s="1" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="K35" s="1" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="L35" s="1" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="M35" s="1" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="N35" s="1" t="n">
+      <c r="B35" s="2" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="C35" s="2" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="D35" s="2" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="E35" s="2" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="F35" s="2" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="G35" s="2" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="H35" s="2" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="I35" s="2" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="J35" s="2" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="K35" s="2" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="L35" s="2" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="M35" s="2" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="N35" s="2" t="n">
         <v>0.98</v>
       </c>
     </row>
@@ -1739,43 +1752,43 @@
           <t>ブロイラー（外部）</t>
         </is>
       </c>
-      <c r="B36" s="1" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="C36" s="1" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="D36" s="1" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="E36" s="1" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="F36" s="1" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="G36" s="1" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="H36" s="1" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="I36" s="1" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="J36" s="1" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="K36" s="1" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="L36" s="1" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="M36" s="1" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="N36" s="1" t="n">
+      <c r="B36" s="2" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="C36" s="2" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="D36" s="2" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="E36" s="2" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="F36" s="2" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="G36" s="2" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="H36" s="2" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="I36" s="2" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="J36" s="2" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="K36" s="2" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="L36" s="2" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="M36" s="2" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="N36" s="2" t="n">
         <v>0.98</v>
       </c>
     </row>
@@ -1785,43 +1798,43 @@
           <t>平均</t>
         </is>
       </c>
-      <c r="B37" s="1" t="n">
+      <c r="B37" s="2" t="n">
         <v>0.9789</v>
       </c>
-      <c r="C37" s="1" t="n">
+      <c r="C37" s="2" t="n">
         <v>0.9789</v>
       </c>
-      <c r="D37" s="1" t="n">
+      <c r="D37" s="2" t="n">
         <v>0.9789</v>
       </c>
-      <c r="E37" s="1" t="n">
+      <c r="E37" s="2" t="n">
         <v>0.9789</v>
       </c>
-      <c r="F37" s="1" t="n">
+      <c r="F37" s="2" t="n">
         <v>0.9789</v>
       </c>
-      <c r="G37" s="1" t="n">
+      <c r="G37" s="2" t="n">
         <v>0.9789</v>
       </c>
-      <c r="H37" s="1" t="n">
+      <c r="H37" s="2" t="n">
         <v>0.9789</v>
       </c>
-      <c r="I37" s="1" t="n">
+      <c r="I37" s="2" t="n">
         <v>0.9789</v>
       </c>
-      <c r="J37" s="1" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="K37" s="1" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="L37" s="1" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="M37" s="1" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="N37" s="1" t="n">
+      <c r="J37" s="2" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="K37" s="2" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="L37" s="2" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="M37" s="2" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="N37" s="2" t="n">
         <v>0.9792999999999999</v>
       </c>
     </row>
@@ -1910,43 +1923,43 @@
           <t>阿波尾鶏</t>
         </is>
       </c>
-      <c r="B41" s="2" t="n">
+      <c r="B41" s="3" t="n">
         <v>3.5</v>
       </c>
-      <c r="C41" s="2" t="n">
+      <c r="C41" s="3" t="n">
         <v>3.5</v>
       </c>
-      <c r="D41" s="2" t="n">
+      <c r="D41" s="3" t="n">
         <v>3.5</v>
       </c>
-      <c r="E41" s="2" t="n">
+      <c r="E41" s="3" t="n">
         <v>3.5</v>
       </c>
-      <c r="F41" s="2" t="n">
+      <c r="F41" s="3" t="n">
         <v>3.5</v>
       </c>
-      <c r="G41" s="2" t="n">
+      <c r="G41" s="3" t="n">
         <v>3.5</v>
       </c>
-      <c r="H41" s="2" t="n">
+      <c r="H41" s="3" t="n">
         <v>3.4</v>
       </c>
-      <c r="I41" s="2" t="n">
+      <c r="I41" s="3" t="n">
         <v>3.4</v>
       </c>
-      <c r="J41" s="2" t="n">
+      <c r="J41" s="3" t="n">
         <v>3.5</v>
       </c>
-      <c r="K41" s="2" t="n">
+      <c r="K41" s="3" t="n">
         <v>3.5</v>
       </c>
-      <c r="L41" s="2" t="n">
+      <c r="L41" s="3" t="n">
         <v>3.5</v>
       </c>
-      <c r="M41" s="2" t="n">
+      <c r="M41" s="3" t="n">
         <v>3.5</v>
       </c>
-      <c r="N41" s="2" t="n">
+      <c r="N41" s="3" t="n">
         <v>3.48</v>
       </c>
     </row>
@@ -1956,43 +1969,43 @@
           <t>赤どり</t>
         </is>
       </c>
-      <c r="B42" s="2" t="n">
+      <c r="B42" s="3" t="n">
         <v>3.1</v>
       </c>
-      <c r="C42" s="2" t="n">
+      <c r="C42" s="3" t="n">
         <v>3.1</v>
       </c>
-      <c r="D42" s="2" t="n">
+      <c r="D42" s="3" t="n">
         <v>3.1</v>
       </c>
-      <c r="E42" s="2" t="n">
+      <c r="E42" s="3" t="n">
         <v>3.1</v>
       </c>
-      <c r="F42" s="2" t="n">
+      <c r="F42" s="3" t="n">
         <v>3.1</v>
       </c>
-      <c r="G42" s="2" t="n">
+      <c r="G42" s="3" t="n">
         <v>3.1</v>
       </c>
-      <c r="H42" s="2" t="n">
+      <c r="H42" s="3" t="n">
         <v>3.1</v>
       </c>
-      <c r="I42" s="2" t="n">
+      <c r="I42" s="3" t="n">
         <v>3.1</v>
       </c>
-      <c r="J42" s="2" t="n">
+      <c r="J42" s="3" t="n">
         <v>3.1</v>
       </c>
-      <c r="K42" s="2" t="n">
+      <c r="K42" s="3" t="n">
         <v>3.1</v>
       </c>
-      <c r="L42" s="2" t="n">
+      <c r="L42" s="3" t="n">
         <v>3.1</v>
       </c>
-      <c r="M42" s="2" t="n">
+      <c r="M42" s="3" t="n">
         <v>3.1</v>
       </c>
-      <c r="N42" s="2" t="n">
+      <c r="N42" s="3" t="n">
         <v>3.1</v>
       </c>
     </row>
@@ -2002,43 +2015,43 @@
           <t>地養鳥</t>
         </is>
       </c>
-      <c r="B43" s="2" t="n">
+      <c r="B43" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="C43" s="2" t="n">
+      <c r="C43" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="D43" s="2" t="n">
+      <c r="D43" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="E43" s="2" t="n">
+      <c r="E43" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="F43" s="2" t="n">
+      <c r="F43" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="G43" s="2" t="n">
+      <c r="G43" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="H43" s="2" t="n">
+      <c r="H43" s="3" t="n">
         <v>2.95</v>
       </c>
-      <c r="I43" s="2" t="n">
+      <c r="I43" s="3" t="n">
         <v>2.95</v>
       </c>
-      <c r="J43" s="2" t="n">
+      <c r="J43" s="3" t="n">
         <v>2.95</v>
       </c>
-      <c r="K43" s="2" t="n">
+      <c r="K43" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="L43" s="2" t="n">
+      <c r="L43" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="M43" s="2" t="n">
+      <c r="M43" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="N43" s="2" t="n">
+      <c r="N43" s="3" t="n">
         <v>2.99</v>
       </c>
     </row>
@@ -2048,43 +2061,43 @@
           <t>ブロイラー</t>
         </is>
       </c>
-      <c r="B44" s="2" t="n">
+      <c r="B44" s="3" t="n">
         <v>3.05</v>
       </c>
-      <c r="C44" s="2" t="n">
+      <c r="C44" s="3" t="n">
         <v>3.05</v>
       </c>
-      <c r="D44" s="2" t="n">
+      <c r="D44" s="3" t="n">
         <v>3.05</v>
       </c>
-      <c r="E44" s="2" t="n">
+      <c r="E44" s="3" t="n">
         <v>3.05</v>
       </c>
-      <c r="F44" s="2" t="n">
+      <c r="F44" s="3" t="n">
         <v>3.05</v>
       </c>
-      <c r="G44" s="2" t="n">
+      <c r="G44" s="3" t="n">
         <v>3.05</v>
       </c>
-      <c r="H44" s="2" t="n">
+      <c r="H44" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="I44" s="2" t="n">
+      <c r="I44" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="J44" s="2" t="n">
+      <c r="J44" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="K44" s="2" t="n">
+      <c r="K44" s="3" t="n">
         <v>3.05</v>
       </c>
-      <c r="L44" s="2" t="n">
+      <c r="L44" s="3" t="n">
         <v>3.05</v>
       </c>
-      <c r="M44" s="2" t="n">
+      <c r="M44" s="3" t="n">
         <v>3.05</v>
       </c>
-      <c r="N44" s="2" t="n">
+      <c r="N44" s="3" t="n">
         <v>3.04</v>
       </c>
     </row>
@@ -2094,43 +2107,43 @@
           <t>ブロイラー（外部）</t>
         </is>
       </c>
-      <c r="B45" s="2" t="n">
+      <c r="B45" s="3" t="n">
         <v>3.05</v>
       </c>
-      <c r="C45" s="2" t="n">
+      <c r="C45" s="3" t="n">
         <v>3.05</v>
       </c>
-      <c r="D45" s="2" t="n">
+      <c r="D45" s="3" t="n">
         <v>3.05</v>
       </c>
-      <c r="E45" s="2" t="n">
+      <c r="E45" s="3" t="n">
         <v>3.05</v>
       </c>
-      <c r="F45" s="2" t="n">
+      <c r="F45" s="3" t="n">
         <v>3.05</v>
       </c>
-      <c r="G45" s="2" t="n">
+      <c r="G45" s="3" t="n">
         <v>3.05</v>
       </c>
-      <c r="H45" s="2" t="n">
+      <c r="H45" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="I45" s="2" t="n">
+      <c r="I45" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="J45" s="2" t="n">
+      <c r="J45" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="K45" s="2" t="n">
+      <c r="K45" s="3" t="n">
         <v>3.05</v>
       </c>
-      <c r="L45" s="2" t="n">
+      <c r="L45" s="3" t="n">
         <v>3.05</v>
       </c>
-      <c r="M45" s="2" t="n">
+      <c r="M45" s="3" t="n">
         <v>3.05</v>
       </c>
-      <c r="N45" s="2" t="n">
+      <c r="N45" s="3" t="n">
         <v>3.04</v>
       </c>
     </row>
@@ -2140,58 +2153,44 @@
           <t>平均</t>
         </is>
       </c>
-      <c r="B46" s="2" t="n">
+      <c r="B46" s="3" t="n">
         <v>3.07</v>
       </c>
-      <c r="C46" s="2" t="n">
+      <c r="C46" s="3" t="n">
         <v>3.07</v>
       </c>
-      <c r="D46" s="2" t="n">
+      <c r="D46" s="3" t="n">
         <v>3.07</v>
       </c>
-      <c r="E46" s="2" t="n">
+      <c r="E46" s="3" t="n">
         <v>3.06</v>
       </c>
-      <c r="F46" s="2" t="n">
+      <c r="F46" s="3" t="n">
         <v>3.07</v>
       </c>
-      <c r="G46" s="2" t="n">
+      <c r="G46" s="3" t="n">
         <v>3.07</v>
       </c>
-      <c r="H46" s="2" t="n">
+      <c r="H46" s="3" t="n">
         <v>3.02</v>
       </c>
-      <c r="I46" s="2" t="n">
+      <c r="I46" s="3" t="n">
         <v>3.02</v>
       </c>
-      <c r="J46" s="2" t="n">
+      <c r="J46" s="3" t="n">
         <v>3.02</v>
       </c>
-      <c r="K46" s="2" t="n">
+      <c r="K46" s="3" t="n">
         <v>3.07</v>
       </c>
-      <c r="L46" s="2" t="n">
+      <c r="L46" s="3" t="n">
         <v>3.07</v>
       </c>
-      <c r="M46" s="2" t="n">
+      <c r="M46" s="3" t="n">
         <v>3.07</v>
       </c>
-      <c r="N46" s="2" t="n">
+      <c r="N46" s="3" t="n">
         <v>3.06</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>出典：アップロードされた「貼り付けたテキスト.txt」の計画欄。空欄・合計・平均は原文どおり。</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>重量の単位は原文の「ｔ」を保持。前回画像の「kg」と表記が異なるため、数値の単位は要確認。単位換算はしていません。</t>
-        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>